<commit_message>
v1.3.6 Corrección extracción de datos de la tabla
</commit_message>
<xml_diff>
--- a/lista_reporte_de_multas_sector_b.xlsx
+++ b/lista_reporte_de_multas_sector_b.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maric\Desktop\auto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A210D755-4524-422D-94B5-68C413163E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E90955-1319-4BA8-B4A2-95B71882C851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2988" yWindow="2100" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LISTA" sheetId="1" r:id="rId1"/>
@@ -283,13 +283,13 @@
     <t>1 EIRL ADVANCED LOGISTICS GROUP (ALG) 20511032114 ADVANC55 ShalomJireh6</t>
   </si>
   <si>
-    <t>EIRL ADVANCED LOGISTICS GROUP (ALG)</t>
-  </si>
-  <si>
-    <t>ADVANC55</t>
-  </si>
-  <si>
-    <t>ShalomJireh6</t>
+    <t>IFTERATC</t>
+  </si>
+  <si>
+    <t>omogonjug</t>
+  </si>
+  <si>
+    <t>GLOVAL SHIPPING LATIN AMERICA (PERU) S.R.L</t>
   </si>
 </sst>
 </file>
@@ -480,8 +480,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1033,20 +1033,20 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="3">
+      <c r="A14" s="26">
         <v>13</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="3">
+        <v>20603083050</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="3">
-        <v>20511032114</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>82</v>
       </c>
       <c r="G14"/>
       <c r="H14"/>

</xml_diff>

<commit_message>
v1.4.0 IMPO235 aereo funcional
</commit_message>
<xml_diff>
--- a/lista_reporte_de_multas_sector_b.xlsx
+++ b/lista_reporte_de_multas_sector_b.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maric\Desktop\auto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E90955-1319-4BA8-B4A2-95B71882C851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FAC318E-85EB-485D-9A34-5DCD4C3CEAEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2988" yWindow="2100" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LISTA" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="82">
   <si>
     <t>NOMBRE</t>
   </si>
@@ -283,20 +283,17 @@
     <t>1 EIRL ADVANCED LOGISTICS GROUP (ALG) 20511032114 ADVANC55 ShalomJireh6</t>
   </si>
   <si>
-    <t>IFTERATC</t>
-  </si>
-  <si>
-    <t>omogonjug</t>
-  </si>
-  <si>
-    <t>GLOVAL SHIPPING LATIN AMERICA (PERU) S.R.L</t>
+    <t>SCHRYVER</t>
+  </si>
+  <si>
+    <t>2024D4rils</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -353,8 +350,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -376,12 +379,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -413,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -478,11 +475,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -763,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.5546875" style="2" customWidth="1"/>
@@ -796,7 +789,7 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="14" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="3">
@@ -1033,14 +1026,14 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="26">
+      <c r="A14" s="3">
         <v>13</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C14" s="3">
-        <v>20603083050</v>
+        <v>20545207436</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>80</v>
@@ -1048,6 +1041,7 @@
       <c r="E14" s="4" t="s">
         <v>81</v>
       </c>
+      <c r="F14"/>
       <c r="G14"/>
       <c r="H14"/>
       <c r="I14"/>
@@ -1114,19 +1108,8 @@
       <c r="J19"/>
       <c r="K19"/>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20"/>
-      <c r="F20"/>
-      <c r="G20"/>
-      <c r="H20"/>
-      <c r="I20"/>
-      <c r="J20"/>
-      <c r="K20"/>
-    </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
@@ -1465,7 +1448,7 @@
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="24" t="s">
         <v>79</v>
       </c>
     </row>

</xml_diff>